<commit_message>
Fix: Reasignar correlativo manual NSGUSD02-014 para Patricia Guzman y documentar en Plan QC
</commit_message>
<xml_diff>
--- a/scratch/TEST_REPORTE_OFICIAL_2026-04-30.xlsx
+++ b/scratch/TEST_REPORTE_OFICIAL_2026-04-30.xlsx
@@ -7368,43 +7368,43 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>NSGUSD02-001.20260314.20260430</t>
+          <t>NSGUSD02-002.20260101.20260430</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Guzmán Manrique Patricia Zarela</t>
+          <t>Schmalhausen Panizo Carla Jeanette</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>20000</v>
+        <v>100000</v>
       </c>
       <c r="E2" t="n">
-        <v>184.11</v>
+        <v>1169.86</v>
       </c>
       <c r="F2" t="n">
-        <v>9.210000000000001</v>
+        <v>58.49</v>
       </c>
       <c r="G2" t="n">
-        <v>174.9</v>
+        <v>1111.37</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>174.9</v>
+        <v>1111.37</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>174.9</v>
+        <v>1111.37</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>20000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="3">
@@ -7413,43 +7413,43 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>NSGUSD02-002.20260101.20260430</t>
+          <t>NSGUSD02-003.20250901.20260430</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Schmalhausen Panizo Carla Jeanette</t>
+          <t>Zavala Távara Piedad Corina</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>100000</v>
+        <v>30000</v>
       </c>
       <c r="E3" t="n">
-        <v>1169.86</v>
+        <v>350.96</v>
       </c>
       <c r="F3" t="n">
-        <v>58.49</v>
+        <v>17.55</v>
       </c>
       <c r="G3" t="n">
-        <v>1111.37</v>
+        <v>333.41</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>1111.37</v>
+        <v>333.41</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>1111.37</v>
+        <v>333.41</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>100000</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="4">
@@ -7458,43 +7458,43 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>NSGUSD02-003.20250901.20260430</t>
+          <t>NSGUSD02-004.20251013.20260430</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Zavala Távara Piedad Corina</t>
+          <t>Lamas Arrasco Angel Eduardo</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>30000</v>
+        <v>102900.26</v>
       </c>
       <c r="E4" t="n">
-        <v>350.96</v>
+        <v>1375.76</v>
       </c>
       <c r="F4" t="n">
-        <v>17.55</v>
+        <v>68.79000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>333.41</v>
+        <v>1306.97</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>1306.97</v>
       </c>
       <c r="I4" t="n">
-        <v>333.41</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>333.41</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>30000</v>
+        <v>104207.23</v>
       </c>
     </row>
     <row r="5">
@@ -7503,43 +7503,43 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NSGUSD02-004.20251013.20260430</t>
+          <t>NSGUSD02-005.20240901.20260430</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Lamas Arrasco Angel Eduardo</t>
+          <t>López Cuellar Greta Yolanda</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>102900.26</v>
+        <v>25584.8</v>
       </c>
       <c r="E5" t="n">
-        <v>1375.76</v>
+        <v>342.07</v>
       </c>
       <c r="F5" t="n">
-        <v>68.79000000000001</v>
+        <v>17.1</v>
       </c>
       <c r="G5" t="n">
-        <v>1306.97</v>
+        <v>324.97</v>
       </c>
       <c r="H5" t="n">
-        <v>1306.97</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>324.97</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>324.97</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>104207.23</v>
+        <v>25584.8</v>
       </c>
     </row>
     <row r="6">
@@ -7548,43 +7548,43 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>NSGUSD02-005.20240901.20260430</t>
+          <t>NSGUSD02-006.20251029.20260430</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>López Cuellar Greta Yolanda</t>
+          <t>Gavidia Cabrera Ernesto Henry</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>25584.8</v>
+        <v>70000</v>
       </c>
       <c r="E6" t="n">
-        <v>342.07</v>
+        <v>994.38</v>
       </c>
       <c r="F6" t="n">
-        <v>17.1</v>
+        <v>49.72</v>
       </c>
       <c r="G6" t="n">
-        <v>324.97</v>
+        <v>944.66</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>324.97</v>
+        <v>944.66</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>324.97</v>
+        <v>944.66</v>
       </c>
       <c r="L6" t="n">
         <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>25584.8</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="7">
@@ -7593,43 +7593,43 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NSGUSD02-006.20251029.20260430</t>
+          <t>NSGUSD02-007.20260104.20260430</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Gavidia Cabrera Ernesto Henry</t>
+          <t>Quintanilla Quispe Asteria Cornelia</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>70000</v>
+        <v>20000</v>
       </c>
       <c r="E7" t="n">
-        <v>994.38</v>
+        <v>267.4</v>
       </c>
       <c r="F7" t="n">
-        <v>49.72</v>
+        <v>13.37</v>
       </c>
       <c r="G7" t="n">
-        <v>944.66</v>
+        <v>254.03</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>944.66</v>
+        <v>254.03</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>944.66</v>
+        <v>254.03</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>70000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="8">
@@ -7638,12 +7638,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>NSGUSD02-007.20260104.20260430</t>
+          <t>NSGUSD02-008.20260203.20260430</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Quintanilla Quispe Asteria Cornelia</t>
+          <t>Quispe Saire Ruth Janet</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -7683,43 +7683,43 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>NSGUSD02-008.20260203.20260430</t>
+          <t>NSGUSD02-009.20260302.20260430</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Quispe Saire Ruth Janet</t>
+          <t>Navarrete  Carlos Alberto</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>20000</v>
+        <v>50000</v>
       </c>
       <c r="E9" t="n">
-        <v>267.4</v>
+        <v>657.53</v>
       </c>
       <c r="F9" t="n">
-        <v>13.37</v>
+        <v>32.88</v>
       </c>
       <c r="G9" t="n">
-        <v>254.03</v>
+        <v>624.65</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>254.03</v>
+        <v>624.65</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>254.03</v>
+        <v>624.65</v>
       </c>
       <c r="L9" t="n">
         <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>20000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="10">
@@ -7728,43 +7728,43 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>NSGUSD02-009.20260302.20260430</t>
+          <t>NSGUSD02-010.20230301.20260430</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Navarrete  Carlos Alberto</t>
+          <t>Gallegos Murga Alejandro Edgar</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="E10" t="n">
-        <v>657.53</v>
+        <v>401.1</v>
       </c>
       <c r="F10" t="n">
-        <v>32.88</v>
+        <v>20.06</v>
       </c>
       <c r="G10" t="n">
-        <v>624.65</v>
+        <v>381.04</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>624.65</v>
+        <v>381.04</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>624.65</v>
+        <v>381.04</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>50000</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="11">
@@ -7773,43 +7773,43 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>NSGUSD02-010.20230301.20260430</t>
+          <t>NSGUSD02-011.20211108.20260430</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Gallegos Murga Alejandro Edgar</t>
+          <t>Villavicencio Bernedo Ricardo Augusto</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>30000</v>
+        <v>20000</v>
       </c>
       <c r="E11" t="n">
-        <v>401.1</v>
+        <v>284.11</v>
       </c>
       <c r="F11" t="n">
-        <v>20.06</v>
+        <v>14.21</v>
       </c>
       <c r="G11" t="n">
-        <v>381.04</v>
+        <v>269.9</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>381.04</v>
+        <v>269.9</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>381.04</v>
+        <v>269.9</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>30000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="12">
@@ -7818,37 +7818,37 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>NSGUSD02-011.20211108.20260430</t>
+          <t>NSGUSD02-012.20260316.20260430</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Villavicencio Bernedo Ricardo Augusto</t>
+          <t>Peñaflor Rivas Eduardo Daniel</t>
         </is>
       </c>
       <c r="D12" t="n">
         <v>20000</v>
       </c>
       <c r="E12" t="n">
-        <v>284.11</v>
+        <v>176.44</v>
       </c>
       <c r="F12" t="n">
-        <v>14.21</v>
+        <v>8.82</v>
       </c>
       <c r="G12" t="n">
-        <v>269.9</v>
+        <v>167.62</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>269.9</v>
+        <v>167.62</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>269.9</v>
+        <v>167.62</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -7863,43 +7863,43 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NSGUSD02-012.20260316.20260430</t>
+          <t>NSGUSD02-013.20260320.20260430</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Peñaflor Rivas Eduardo Daniel</t>
+          <t>Mc Iver Donald Angus</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>20000</v>
+        <v>50000</v>
       </c>
       <c r="E13" t="n">
-        <v>176.44</v>
+        <v>460.27</v>
       </c>
       <c r="F13" t="n">
-        <v>8.82</v>
+        <v>23.01</v>
       </c>
       <c r="G13" t="n">
-        <v>167.62</v>
+        <v>437.26</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>437.26</v>
       </c>
       <c r="I13" t="n">
-        <v>167.62</v>
+        <v>0</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>167.62</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>20000</v>
+        <v>50437.26</v>
       </c>
     </row>
     <row r="14">
@@ -7908,43 +7908,43 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>NSGUSD02-013.20260320.20260430</t>
+          <t>NSGUSD02-014.20260314.20260430</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Mc Iver Donald Angus</t>
+          <t>Guzmán Manrique Patricia Zarela</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>50000</v>
+        <v>20000</v>
       </c>
       <c r="E14" t="n">
-        <v>460.27</v>
+        <v>184.11</v>
       </c>
       <c r="F14" t="n">
-        <v>23.01</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="G14" t="n">
-        <v>437.26</v>
+        <v>174.9</v>
       </c>
       <c r="H14" t="n">
-        <v>437.26</v>
+        <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>174.9</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>174.9</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>50437.26</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="15">

</xml_diff>